<commit_message>
Automatiza 114 arquivo(s) de processos no backend
</commit_message>
<xml_diff>
--- a/planilhas/LISTA DE PROCESSO PG + ECO HIBRIDO LADO MENOR.xlsx
+++ b/planilhas/LISTA DE PROCESSO PG + ECO HIBRIDO LADO MENOR.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" state="visible" r:id="rId1"/>
@@ -1460,7 +1460,7 @@
         <v/>
       </c>
       <c r="E39" t="n">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
@@ -1489,7 +1489,7 @@
         <v/>
       </c>
       <c r="E40" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
@@ -1518,7 +1518,7 @@
         <v/>
       </c>
       <c r="E41" t="n">
-        <v>4</v>
+        <v>41</v>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
@@ -1547,7 +1547,7 @@
         <v/>
       </c>
       <c r="E42" t="n">
-        <v>1</v>
+        <v>158</v>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
@@ -1576,7 +1576,7 @@
         <v/>
       </c>
       <c r="E43" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
@@ -1605,7 +1605,7 @@
         <v/>
       </c>
       <c r="E44" t="n">
-        <v>3</v>
+        <v>34</v>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
@@ -1634,7 +1634,7 @@
         <v/>
       </c>
       <c r="E45" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
@@ -1663,7 +1663,7 @@
         <v/>
       </c>
       <c r="E46" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>

</xml_diff>